<commit_message>
update logic and viewer
</commit_message>
<xml_diff>
--- a/class.xlsx
+++ b/class.xlsx
@@ -723,574 +723,574 @@
   </cols>
   <sheetData>
     <row r="1" ht="18.95" customHeight="1" s="7">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="0" t="inlineStr">
         <is>
           <t>优先级</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="0" t="inlineStr">
         <is>
           <t>一级分类</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="0" t="inlineStr">
         <is>
           <t>二级分类</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="0" t="inlineStr">
         <is>
           <t>名称</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="0" t="inlineStr">
         <is>
           <t>缩写</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="0" t="inlineStr">
         <is>
           <t>特征及判据</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18.95" customHeight="1" s="7">
-      <c r="A2" t="n">
+      <c r="A2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="0" t="inlineStr">
         <is>
           <t>BLOCK</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="0" t="inlineStr">
         <is>
           <t>宏块</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="0" t="inlineStr">
         <is>
           <t>MACRO_BLOCK</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="0" t="inlineStr">
         <is>
           <t>MBLK</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="0" t="inlineStr">
         <is>
           <t>连通域 fail bit 数 / macro 总 bit 数（如 ≥30%）</t>
         </is>
       </c>
     </row>
     <row r="3" ht="33.95" customHeight="1" s="7">
-      <c r="A3" t="n">
+      <c r="A3" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="0" t="inlineStr">
         <is>
           <t>LINE-ROW</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="0" t="inlineStr">
         <is>
           <t>单行</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="0" t="inlineStr">
         <is>
           <t>SWR</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="0" t="inlineStr">
         <is>
           <t>SWR</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="0" t="inlineStr">
         <is>
           <t>同一 WL 上 fail 数 / 总 BL 数 ≥ 40%</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18.95" customHeight="1" s="7">
-      <c r="A4" t="n">
+      <c r="A4" s="0" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="0" t="inlineStr">
         <is>
           <t>LINE-COLUMN</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="0" t="inlineStr">
         <is>
           <t>单列</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="0" t="inlineStr">
         <is>
           <t>SBC</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="0" t="inlineStr">
         <is>
           <t>SBC</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="0" t="inlineStr">
         <is>
           <t>同一 BL 上 fail 数 / 总 WL 数 ≥ 40%</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18.95" customHeight="1" s="7">
-      <c r="A5" t="n">
+      <c r="A5" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="0" t="inlineStr">
         <is>
           <t>LINE-ROW</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="0" t="inlineStr">
         <is>
           <t>部分行</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="0" t="inlineStr">
         <is>
           <t>PWR</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="0" t="inlineStr">
         <is>
           <t>PWR</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="0" t="inlineStr">
         <is>
           <t>同一 WL 上存在连续 fail，连续长度 L &gt; 20，且该 WL fail 占比 &lt; 40%</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18.95" customHeight="1" s="7">
-      <c r="A6" t="n">
+      <c r="A6" s="0" t="n">
         <v>4</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="0" t="inlineStr">
         <is>
           <t>LINE-COLUMN</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="0" t="inlineStr">
         <is>
           <t>部分列</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="0" t="inlineStr">
         <is>
           <t>PBC</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="0" t="inlineStr">
         <is>
           <t>PBC</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="0" t="inlineStr">
         <is>
           <t>同一 BL 上存在连续 fail，连续长度 L &gt; 20，且该 BL fail 占比 &lt; 40%</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18.95" customHeight="1" s="7">
-      <c r="A7" t="n">
+      <c r="A7" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="0" t="inlineStr">
         <is>
           <t>LINE-ROW</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="0" t="inlineStr">
         <is>
           <t>多行</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="0" t="inlineStr">
         <is>
           <t>MWR</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="0" t="inlineStr">
         <is>
           <t>MWR</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="0" t="inlineStr">
         <is>
           <t>≥2 条相邻 WL 分别满足 SWR 或 PWR，表示多行方向异常</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18.95" customHeight="1" s="7">
-      <c r="A8" t="n">
+      <c r="A8" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="0" t="inlineStr">
         <is>
           <t>LINE-COLUMN</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="0" t="inlineStr">
         <is>
           <t>多列</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="0" t="inlineStr">
         <is>
           <t>MBC</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E8" s="0" t="inlineStr">
         <is>
           <t>MBC</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="0" t="inlineStr">
         <is>
           <t>≥2 条相邻 BL 分别满足 SBC 或 PBC，表示多列方向异常</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18.95" customHeight="1" s="7">
-      <c r="A9" t="n">
+      <c r="A9" s="0" t="n">
         <v>6</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>CROSS</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="0" t="inlineStr">
         <is>
           <t>交叉</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="0" t="inlineStr">
         <is>
           <t>CROSS</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E9" s="0" t="inlineStr">
         <is>
           <t>CRS</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>SWR/PWR/MWR 任一个与 SBC/PBC/MBC 任一个同时存在且相交</t>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t>SWR/PWR/MWR 与 SBC/PBC/MBC 存在真实交叉；交叉点左右、上下两侧 arm 长度均需 &gt;= cross_min_arm_len（默认 20），共享线段或点集的多个交叉会合并为同一个 CROSS id</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18.95" customHeight="1" s="7">
-      <c r="A10" t="n">
+      <c r="A10" s="0" t="n">
         <v>7</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="0" t="inlineStr">
         <is>
           <t>BLOCK</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="0" t="inlineStr">
         <is>
           <t>块</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="0" t="inlineStr">
         <is>
           <t>BLOCK</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E10" s="0" t="inlineStr">
         <is>
           <t>BLK</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" s="0" t="inlineStr">
         <is>
           <t>连通域 size ≥ 阈值（如≥25）, 0.8 &lt; 行范围/列范围 &lt; 1.2，且填充占行列范围之比 &gt; 60%</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18.95" customHeight="1" s="7">
-      <c r="A11" t="n">
+      <c r="A11" s="0" t="n">
         <v>8</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="0" t="inlineStr">
         <is>
           <t>BLOCK</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="0" t="inlineStr">
         <is>
           <t>四点块</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="0" t="inlineStr">
         <is>
           <t>QUADRA_BIT</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E11" s="0" t="inlineStr">
         <is>
           <t>QB</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="0" t="inlineStr">
         <is>
           <t>连通域 size=4 且 bounding box=2×2 且完全填充</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18.95" customHeight="1" s="7">
-      <c r="A12" t="n">
+      <c r="A12" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="0" t="inlineStr">
         <is>
           <t>RANDOM</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="0" t="inlineStr">
         <is>
           <t>随机簇</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="0" t="inlineStr">
         <is>
           <t>RANDOM_CLUSTER</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E12" s="0" t="inlineStr">
         <is>
           <t>RCLU</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" s="0" t="inlineStr">
         <is>
           <t>连通域 size ≥3 且不满足行/列/quadra/block/TB 结构</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18.95" customHeight="1" s="7">
-      <c r="A13" t="n">
+      <c r="A13" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="0" t="inlineStr">
         <is>
           <t>LINE-ROW</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="0" t="inlineStr">
         <is>
           <t>点状行</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="0" t="inlineStr">
         <is>
           <t>DOTTED_ROW</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E13" s="0" t="inlineStr">
         <is>
           <t>DWR</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="0" t="inlineStr">
         <is>
           <t>同一或多个相邻 WL 内，存在多个不连续 fail component，点数 &gt;=6，横向 span &gt;=20，且最大连续段 &lt;= PWR 阈值；视觉上呈点状行 failure。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="33" customHeight="1" s="7">
-      <c r="A14" t="n">
+      <c r="A14" s="0" t="n">
         <v>9</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>LINE-COLUMN</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="0" t="inlineStr">
         <is>
           <t>点状列</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="0" t="inlineStr">
         <is>
           <t>DOTTED_COLUMN</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E14" s="0" t="inlineStr">
         <is>
           <t>DWC</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" s="0" t="inlineStr">
         <is>
           <t>同一或多个相邻 BL 内，存在多个不连续 fail component，点数 &gt;=6，纵向 span &gt;=20，且最大连续段 &lt;= PBC 阈值；视觉上呈点状列 failure。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="33" customHeight="1" s="7">
-      <c r="A15" t="n">
+      <c r="A15" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="0" t="inlineStr">
         <is>
           <t>SINGLE</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="0" t="inlineStr">
         <is>
           <t>单点</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="0" t="inlineStr">
         <is>
           <t>SB</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E15" s="0" t="inlineStr">
         <is>
           <t>SB</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" s="0" t="inlineStr">
         <is>
           <t>连通域 size = 1；邻域（如3×3）内无其他 fail</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18.95" customHeight="1" s="7">
-      <c r="A16" t="n">
+      <c r="A16" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>LINE-DOUBLE</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="0" t="inlineStr">
         <is>
           <t>双行</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="0" t="inlineStr">
         <is>
           <t>DBR</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="0" t="inlineStr">
         <is>
           <t>DBR</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" s="0" t="inlineStr">
         <is>
           <t>同一 WL 相邻的两个 Bit fail</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18.95" customHeight="1" s="7">
-      <c r="A17" t="n">
+      <c r="A17" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="0" t="inlineStr">
         <is>
           <t>LINE-DOUBLE</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="0" t="inlineStr">
         <is>
           <t>双列</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="0" t="inlineStr">
         <is>
           <t>DBC</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="0" t="inlineStr">
         <is>
           <t>DBC</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" s="0" t="inlineStr">
         <is>
           <t>同一 BL 相邻的两个 Bit fail</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18.95" customHeight="1" s="7">
-      <c r="A18" t="n">
+      <c r="A18" s="0" t="n">
         <v>10</v>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="0" t="inlineStr">
         <is>
           <t>TB</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="0" t="inlineStr">
         <is>
           <t>三点弯折</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="0" t="inlineStr">
         <is>
           <t>TB</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="0" t="inlineStr">
         <is>
           <t>TB</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" s="0" t="inlineStr">
         <is>
           <t>三点 L 形</t>
         </is>
       </c>
     </row>
     <row r="19" ht="16.5" customHeight="1" s="7">
-      <c r="A19" t="n">
+      <c r="A19" s="0" t="n">
         <v>11</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="0" t="inlineStr">
         <is>
           <t>RANDOM</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="0" t="inlineStr">
         <is>
           <t>整体随机</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="0" t="inlineStr">
         <is>
           <t>RANDOM_DENSITY</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E19" s="0" t="inlineStr">
         <is>
           <t>RDEN</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>同一个 MACRO 存在大量的 SB/DBR/DBC/QB/TB/RANDOM_CLUSTER，超过 200 个；这些小 mode 的类型会被 RDEN 覆盖</t>
+      <c r="F19" s="0" t="inlineStr">
+        <is>
+          <t>同一个 MACRO 中 SB/DBR/DBC/QB/TB/RANDOM_CLUSTER/DOTTED_ROW/DOTTED_COLUMN 会先按 bbox 间距 &lt;=100 分成相邻组；同一组的 pattern 数量或 fail bit 数量超过 200，且该组覆盖范围 x_span 与 y_span 均 &gt; macro 对应方向 30%，这些 mode 才会被 RDEN 覆盖。远离该组超过 100 的点不参与该组统计。</t>
         </is>
       </c>
     </row>

</xml_diff>